<commit_message>
docs: add readme, fix tender sync paths, and migrate secrets to monorepo
- Created a comprehensive README.md.
- Fixed directory paths in `md_to_excel.py`, `tender_sync_api.py`, and `registry-sync-excel.yml` (removed 'opportunities/' prefix).
- Created `tender-sync.yml` to automate daily tender fetching.
- Updated `md_to_excel.py` to only include verified/active data in Excel exports.
- Updated `agent-automated.yml` and `registry-weekly-report.yml` to fetch `production.env` from the RokctAI/Monorepo using the GitHub CLI.
</commit_message>
<xml_diff>
--- a/published/01_Equity_Africa.xlsx
+++ b/published/01_Equity_Africa.xlsx
@@ -19,16 +19,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -55,7 +52,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -63,19 +60,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -526,33 +517,33 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Partech</t>
+          <t>Future Africa</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Philippe Collombel</t>
+          <t>Iyinoluwa Aboyeji</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/philippecollombel</t>
+          <t>https://www.linkedin.com/in/eaboyeji/</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[partechpartners.com](https://partechpartners.com)</t>
+          <t>[future.africa](https://www.future.africa)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Europe / Africa</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -567,55 +558,51 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Seed / Series A-Z</t>
+          <t>Seed / Series A</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>[Team/Contact](https://partechpartners.com/team/)</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>Strong Africa presence</t>
-        </is>
-      </c>
+          <t>https://www.future.africa/about-us</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Norrsken VC</t>
+          <t>Ventures Platform</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Niklas Adalberth</t>
+          <t>Kola Aina</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/niklas-adalberth</t>
+          <t>https://www.linkedin.com/in/kola-aina-vp/</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>[norrsken.vc](https://norrsken.vc)</t>
+          <t>[venturesplatform.com](https://www.venturesplatform.com)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Europe / Africa</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Tech / Impact / Emerging Markets</t>
+          <t>Tech / Fintech</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -630,50 +617,46 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>[Team/Contact](https://norrsken.vc/about)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Impact investing</t>
-        </is>
-      </c>
+          <t>https://www.venturesplatform.com/team</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>CRE Venture Capital</t>
+          <t>EchoVC</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Pardon Makumbe</t>
+          <t>Eghosa Omoigui</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/pardonmakumbe</t>
+          <t>https://www.linkedin.com/pub/eghosa-omoigui/0/a/888</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>[cre.vc](https://cre.vc)</t>
+          <t>[echovc.com](https://www.echovc.com)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>Africa / Emerging Markets</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Tech / Emerging Markets</t>
+          <t>Tech</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -683,45 +666,41 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Seed / Series A</t>
+          <t>Seed / Early Stage</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>[Team/Contact](https://cre.vc)</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>Sub-Saharan Africa focus</t>
-        </is>
-      </c>
+          <t>https://www.echovc.com/team</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TLcom Capital</t>
+          <t>Launch Africa</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Maurizio Caio</t>
+          <t>Zachariah George</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/mauriziocaio</t>
+          <t>https://www.linkedin.com/in/zachariahgeorge/</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>[tlcomcapital.com](https://tlcomcapital.com)</t>
+          <t>[launchafrica.vc](https://launchafrica.vc)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>UK / Kenya</t>
+          <t>Mauritius</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -741,40 +720,36 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Seed / Series A-Z</t>
+          <t>Seed / Pre-Series A</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>[Team/Contact](https://tlcomcapital.com/team/)</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>African tech ecosystem</t>
-        </is>
-      </c>
+          <t>https://www.launchafrica.vc/team</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Novastar Ventures</t>
+          <t>Savannah Fund</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Steve Beck</t>
+          <t>Mbwana Alliy</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/stevebeck</t>
+          <t>https://www.linkedin.com/in/mbwana/</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>[novastarventures.com](https://novastarventures.com)</t>
+          <t>[savannah.vc](https://savannah.vc)</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -789,7 +764,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Tech / Emerging Markets</t>
+          <t>Tech</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -799,50 +774,46 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Seed / Series A</t>
+          <t>Seed</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>[Team/Contact](https://novastarventures.com/team/)</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>East and West Africa</t>
-        </is>
-      </c>
+          <t>https://savannah.vc/team</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Flat6Labs</t>
+          <t>Partech</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Ramez El-Serafy</t>
+          <t>Philippe Collombel</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/ramezelserafy</t>
+          <t>https://www.linkedin.com/in/philippecollombel</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>[flat6labs.com](https://flat6labs.com)</t>
+          <t>[partechpartners.com](https://partechpartners.com)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>France</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>MENA</t>
+          <t>Europe / Africa</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -852,60 +823,60 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>VC/Accelerator</t>
+          <t>VC</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Pre-Seed / Seed</t>
+          <t>Seed / Series A-Z</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>[Team/Contact](https://flat6labs.com/about/)</t>
+          <t>[Team/Contact](https://partechpartners.com/team/)</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>MENA region focus</t>
+          <t>Strong Africa presence</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Future Africa</t>
+          <t>Norrsken VC</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Iyinoluwa Aboyeji</t>
+          <t>Niklas Adalberth</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/eaboyeji/</t>
+          <t>https://www.linkedin.com/in/niklas-adalberth</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>[future.africa](https://www.future.africa)</t>
+          <t>[norrsken.vc](https://norrsken.vc)</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>Europe / Africa</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Tech / Emerging Markets</t>
+          <t>Tech / Impact / Emerging Markets</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -920,36 +891,40 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>https://www.future.africa/about-us</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr"/>
+          <t>[Team/Contact](https://norrsken.vc/about)</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Impact investing</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Ventures Platform</t>
+          <t>CRE Venture Capital</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Kola Aina</t>
+          <t>Pardon Makumbe</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/kola-aina-vp/</t>
+          <t>https://www.linkedin.com/in/pardonmakumbe</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>[venturesplatform.com](https://www.venturesplatform.com)</t>
+          <t>[cre.vc](https://cre.vc)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -959,7 +934,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Tech / Fintech</t>
+          <t>Tech / Emerging Markets</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -974,46 +949,50 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>https://www.venturesplatform.com/team</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr"/>
+          <t>[Team/Contact](https://cre.vc)</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Sub-Saharan Africa focus</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>EchoVC</t>
+          <t>TLcom Capital</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Eghosa Omoigui</t>
+          <t>Maurizio Caio</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/pub/eghosa-omoigui/0/a/888</t>
+          <t>https://www.linkedin.com/in/mauriziocaio</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>[echovc.com](https://www.echovc.com)</t>
+          <t>[tlcomcapital.com](https://tlcomcapital.com)</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>UK / Kenya</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Africa / Emerging Markets</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Tech</t>
+          <t>Tech / Emerging Markets</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -1023,41 +1002,45 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Seed / Early Stage</t>
+          <t>Seed / Series A-Z</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>https://www.echovc.com/team</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr"/>
+          <t>[Team/Contact](https://tlcomcapital.com/team/)</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>African tech ecosystem</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Launch Africa</t>
+          <t>Novastar Ventures</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Zachariah George</t>
+          <t>Steve Beck</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/zachariahgeorge/</t>
+          <t>https://www.linkedin.com/in/stevebeck</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>[launchafrica.vc](https://launchafrica.vc)</t>
+          <t>[novastarventures.com](https://novastarventures.com)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Mauritius</t>
+          <t>Kenya</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1077,69 +1060,77 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Seed / Pre-Series A</t>
+          <t>Seed / Series A</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>https://www.launchafrica.vc/team</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr"/>
+          <t>[Team/Contact](https://novastarventures.com/team/)</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>East and West Africa</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Savannah Fund</t>
+          <t>Flat6Labs</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Mbwana Alliy</t>
+          <t>Ramez El-Serafy</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/mbwana/</t>
+          <t>https://www.linkedin.com/in/ramezelserafy</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>[savannah.vc](https://savannah.vc)</t>
+          <t>[flat6labs.com](https://flat6labs.com)</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Kenya</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>MENA</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Tech</t>
+          <t>Tech / Emerging Markets</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>VC</t>
+          <t>VC/Accelerator</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Seed</t>
+          <t>Pre-Seed / Seed</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>https://savannah.vc/team</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr"/>
+          <t>[Team/Contact](https://flat6labs.com/about/)</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>MENA region focus</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:L12"/>

</xml_diff>

<commit_message>
docs: add README, fix tender sync paths, and migrate secrets
- Added a comprehensive README.md.
- Fixed directory paths in sync scripts and workflows (removed 'opportunities/' prefix).
- Created 'tender-sync.yml' for daily automated tender fetching.
- Updated 'md_to_excel.py' to only include verified/active data in exports.
- Migrated secret handling to fetch 'production.env' from Monorepo via 'gh api' for better security and consistency.
</commit_message>
<xml_diff>
--- a/published/01_Equity_Africa.xlsx
+++ b/published/01_Equity_Africa.xlsx
@@ -19,16 +19,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -55,7 +52,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -63,19 +60,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -526,33 +517,33 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Partech</t>
+          <t>Future Africa</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Philippe Collombel</t>
+          <t>Iyinoluwa Aboyeji</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/philippecollombel</t>
+          <t>https://www.linkedin.com/in/eaboyeji/</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[partechpartners.com](https://partechpartners.com)</t>
+          <t>[future.africa](https://www.future.africa)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Europe / Africa</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -567,55 +558,51 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Seed / Series A-Z</t>
+          <t>Seed / Series A</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>[Team/Contact](https://partechpartners.com/team/)</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>Strong Africa presence</t>
-        </is>
-      </c>
+          <t>https://www.future.africa/about-us</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Norrsken VC</t>
+          <t>Ventures Platform</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Niklas Adalberth</t>
+          <t>Kola Aina</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/niklas-adalberth</t>
+          <t>https://www.linkedin.com/in/kola-aina-vp/</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>[norrsken.vc](https://norrsken.vc)</t>
+          <t>[venturesplatform.com](https://www.venturesplatform.com)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Europe / Africa</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Tech / Impact / Emerging Markets</t>
+          <t>Tech / Fintech</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -630,50 +617,46 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>[Team/Contact](https://norrsken.vc/about)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Impact investing</t>
-        </is>
-      </c>
+          <t>https://www.venturesplatform.com/team</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>CRE Venture Capital</t>
+          <t>EchoVC</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Pardon Makumbe</t>
+          <t>Eghosa Omoigui</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/pardonmakumbe</t>
+          <t>https://www.linkedin.com/pub/eghosa-omoigui/0/a/888</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>[cre.vc](https://cre.vc)</t>
+          <t>[echovc.com](https://www.echovc.com)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>Africa / Emerging Markets</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Tech / Emerging Markets</t>
+          <t>Tech</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -683,45 +666,41 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Seed / Series A</t>
+          <t>Seed / Early Stage</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>[Team/Contact](https://cre.vc)</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>Sub-Saharan Africa focus</t>
-        </is>
-      </c>
+          <t>https://www.echovc.com/team</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TLcom Capital</t>
+          <t>Launch Africa</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Maurizio Caio</t>
+          <t>Zachariah George</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/mauriziocaio</t>
+          <t>https://www.linkedin.com/in/zachariahgeorge/</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>[tlcomcapital.com](https://tlcomcapital.com)</t>
+          <t>[launchafrica.vc](https://launchafrica.vc)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>UK / Kenya</t>
+          <t>Mauritius</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -741,40 +720,36 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Seed / Series A-Z</t>
+          <t>Seed / Pre-Series A</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>[Team/Contact](https://tlcomcapital.com/team/)</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>African tech ecosystem</t>
-        </is>
-      </c>
+          <t>https://www.launchafrica.vc/team</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Novastar Ventures</t>
+          <t>Savannah Fund</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Steve Beck</t>
+          <t>Mbwana Alliy</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/stevebeck</t>
+          <t>https://www.linkedin.com/in/mbwana/</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>[novastarventures.com](https://novastarventures.com)</t>
+          <t>[savannah.vc](https://savannah.vc)</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -789,7 +764,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Tech / Emerging Markets</t>
+          <t>Tech</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -799,50 +774,46 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Seed / Series A</t>
+          <t>Seed</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>[Team/Contact](https://novastarventures.com/team/)</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>East and West Africa</t>
-        </is>
-      </c>
+          <t>https://savannah.vc/team</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Flat6Labs</t>
+          <t>Partech</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Ramez El-Serafy</t>
+          <t>Philippe Collombel</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/ramezelserafy</t>
+          <t>https://www.linkedin.com/in/philippecollombel</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>[flat6labs.com](https://flat6labs.com)</t>
+          <t>[partechpartners.com](https://partechpartners.com)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>France</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>MENA</t>
+          <t>Europe / Africa</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -852,60 +823,60 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>VC/Accelerator</t>
+          <t>VC</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Pre-Seed / Seed</t>
+          <t>Seed / Series A-Z</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>[Team/Contact](https://flat6labs.com/about/)</t>
+          <t>[Team/Contact](https://partechpartners.com/team/)</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>MENA region focus</t>
+          <t>Strong Africa presence</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Future Africa</t>
+          <t>Norrsken VC</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Iyinoluwa Aboyeji</t>
+          <t>Niklas Adalberth</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/eaboyeji/</t>
+          <t>https://www.linkedin.com/in/niklas-adalberth</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>[future.africa](https://www.future.africa)</t>
+          <t>[norrsken.vc](https://norrsken.vc)</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>Europe / Africa</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Tech / Emerging Markets</t>
+          <t>Tech / Impact / Emerging Markets</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -920,36 +891,40 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>https://www.future.africa/about-us</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr"/>
+          <t>[Team/Contact](https://norrsken.vc/about)</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Impact investing</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Ventures Platform</t>
+          <t>CRE Venture Capital</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Kola Aina</t>
+          <t>Pardon Makumbe</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/kola-aina-vp/</t>
+          <t>https://www.linkedin.com/in/pardonmakumbe</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>[venturesplatform.com](https://www.venturesplatform.com)</t>
+          <t>[cre.vc](https://cre.vc)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -959,7 +934,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Tech / Fintech</t>
+          <t>Tech / Emerging Markets</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -974,46 +949,50 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>https://www.venturesplatform.com/team</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr"/>
+          <t>[Team/Contact](https://cre.vc)</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Sub-Saharan Africa focus</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>EchoVC</t>
+          <t>TLcom Capital</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Eghosa Omoigui</t>
+          <t>Maurizio Caio</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/pub/eghosa-omoigui/0/a/888</t>
+          <t>https://www.linkedin.com/in/mauriziocaio</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>[echovc.com](https://www.echovc.com)</t>
+          <t>[tlcomcapital.com](https://tlcomcapital.com)</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>UK / Kenya</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Africa / Emerging Markets</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Tech</t>
+          <t>Tech / Emerging Markets</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -1023,41 +1002,45 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Seed / Early Stage</t>
+          <t>Seed / Series A-Z</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>https://www.echovc.com/team</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr"/>
+          <t>[Team/Contact](https://tlcomcapital.com/team/)</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>African tech ecosystem</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Launch Africa</t>
+          <t>Novastar Ventures</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Zachariah George</t>
+          <t>Steve Beck</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/zachariahgeorge/</t>
+          <t>https://www.linkedin.com/in/stevebeck</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>[launchafrica.vc](https://launchafrica.vc)</t>
+          <t>[novastarventures.com](https://novastarventures.com)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Mauritius</t>
+          <t>Kenya</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1077,69 +1060,77 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Seed / Pre-Series A</t>
+          <t>Seed / Series A</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>https://www.launchafrica.vc/team</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr"/>
+          <t>[Team/Contact](https://novastarventures.com/team/)</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>East and West Africa</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Savannah Fund</t>
+          <t>Flat6Labs</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Mbwana Alliy</t>
+          <t>Ramez El-Serafy</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/mbwana/</t>
+          <t>https://www.linkedin.com/in/ramezelserafy</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>[savannah.vc](https://savannah.vc)</t>
+          <t>[flat6labs.com](https://flat6labs.com)</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Kenya</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>MENA</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Tech</t>
+          <t>Tech / Emerging Markets</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>VC</t>
+          <t>VC/Accelerator</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Seed</t>
+          <t>Pre-Seed / Seed</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>https://savannah.vc/team</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr"/>
+          <t>[Team/Contact](https://flat6labs.com/about/)</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>MENA region focus</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:L12"/>

</xml_diff>

<commit_message>
fix: add README, fix tender sync, migrate secrets, and update permissions
- Created a comprehensive README.md.
- Corrected directory paths in sync scripts and workflows (removed 'opportunities/' prefix).
- Created 'tender-sync.yml' for daily automated tender sync.
- Updated 'md_to_excel.py' to include only verified/active data in exports.
- Migrated secret management to fetch 'production.env' from Monorepo via 'gh api'.
- Added 'permissions: write-all' to workflows that modify files.
</commit_message>
<xml_diff>
--- a/published/01_Equity_Africa.xlsx
+++ b/published/01_Equity_Africa.xlsx
@@ -19,16 +19,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -55,7 +52,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -63,19 +60,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -526,33 +517,33 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Partech</t>
+          <t>Future Africa</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Philippe Collombel</t>
+          <t>Iyinoluwa Aboyeji</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/philippecollombel</t>
+          <t>https://www.linkedin.com/in/eaboyeji/</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[partechpartners.com](https://partechpartners.com)</t>
+          <t>[future.africa](https://www.future.africa)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Europe / Africa</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -567,55 +558,51 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Seed / Series A-Z</t>
+          <t>Seed / Series A</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>[Team/Contact](https://partechpartners.com/team/)</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>Strong Africa presence</t>
-        </is>
-      </c>
+          <t>https://www.future.africa/about-us</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Norrsken VC</t>
+          <t>Ventures Platform</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Niklas Adalberth</t>
+          <t>Kola Aina</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/niklas-adalberth</t>
+          <t>https://www.linkedin.com/in/kola-aina-vp/</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>[norrsken.vc](https://norrsken.vc)</t>
+          <t>[venturesplatform.com](https://www.venturesplatform.com)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Europe / Africa</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Tech / Impact / Emerging Markets</t>
+          <t>Tech / Fintech</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -630,50 +617,46 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>[Team/Contact](https://norrsken.vc/about)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Impact investing</t>
-        </is>
-      </c>
+          <t>https://www.venturesplatform.com/team</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>CRE Venture Capital</t>
+          <t>EchoVC</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Pardon Makumbe</t>
+          <t>Eghosa Omoigui</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/pardonmakumbe</t>
+          <t>https://www.linkedin.com/pub/eghosa-omoigui/0/a/888</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>[cre.vc](https://cre.vc)</t>
+          <t>[echovc.com](https://www.echovc.com)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>Africa / Emerging Markets</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Tech / Emerging Markets</t>
+          <t>Tech</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -683,45 +666,41 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Seed / Series A</t>
+          <t>Seed / Early Stage</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>[Team/Contact](https://cre.vc)</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>Sub-Saharan Africa focus</t>
-        </is>
-      </c>
+          <t>https://www.echovc.com/team</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TLcom Capital</t>
+          <t>Launch Africa</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Maurizio Caio</t>
+          <t>Zachariah George</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/mauriziocaio</t>
+          <t>https://www.linkedin.com/in/zachariahgeorge/</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>[tlcomcapital.com](https://tlcomcapital.com)</t>
+          <t>[launchafrica.vc](https://launchafrica.vc)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>UK / Kenya</t>
+          <t>Mauritius</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -741,40 +720,36 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Seed / Series A-Z</t>
+          <t>Seed / Pre-Series A</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>[Team/Contact](https://tlcomcapital.com/team/)</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>African tech ecosystem</t>
-        </is>
-      </c>
+          <t>https://www.launchafrica.vc/team</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Novastar Ventures</t>
+          <t>Savannah Fund</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Steve Beck</t>
+          <t>Mbwana Alliy</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/stevebeck</t>
+          <t>https://www.linkedin.com/in/mbwana/</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>[novastarventures.com](https://novastarventures.com)</t>
+          <t>[savannah.vc](https://savannah.vc)</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -789,7 +764,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Tech / Emerging Markets</t>
+          <t>Tech</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -799,50 +774,46 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Seed / Series A</t>
+          <t>Seed</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>[Team/Contact](https://novastarventures.com/team/)</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>East and West Africa</t>
-        </is>
-      </c>
+          <t>https://savannah.vc/team</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Flat6Labs</t>
+          <t>Partech</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Ramez El-Serafy</t>
+          <t>Philippe Collombel</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/ramezelserafy</t>
+          <t>https://www.linkedin.com/in/philippecollombel</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>[flat6labs.com](https://flat6labs.com)</t>
+          <t>[partechpartners.com](https://partechpartners.com)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>France</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>MENA</t>
+          <t>Europe / Africa</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -852,60 +823,60 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>VC/Accelerator</t>
+          <t>VC</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Pre-Seed / Seed</t>
+          <t>Seed / Series A-Z</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>[Team/Contact](https://flat6labs.com/about/)</t>
+          <t>[Team/Contact](https://partechpartners.com/team/)</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>MENA region focus</t>
+          <t>Strong Africa presence</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Future Africa</t>
+          <t>Norrsken VC</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Iyinoluwa Aboyeji</t>
+          <t>Niklas Adalberth</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/eaboyeji/</t>
+          <t>https://www.linkedin.com/in/niklas-adalberth</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>[future.africa](https://www.future.africa)</t>
+          <t>[norrsken.vc](https://norrsken.vc)</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>Europe / Africa</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Tech / Emerging Markets</t>
+          <t>Tech / Impact / Emerging Markets</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -920,36 +891,40 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>https://www.future.africa/about-us</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr"/>
+          <t>[Team/Contact](https://norrsken.vc/about)</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Impact investing</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Ventures Platform</t>
+          <t>CRE Venture Capital</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Kola Aina</t>
+          <t>Pardon Makumbe</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/kola-aina-vp/</t>
+          <t>https://www.linkedin.com/in/pardonmakumbe</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>[venturesplatform.com](https://www.venturesplatform.com)</t>
+          <t>[cre.vc](https://cre.vc)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -959,7 +934,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Tech / Fintech</t>
+          <t>Tech / Emerging Markets</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -974,46 +949,50 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>https://www.venturesplatform.com/team</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr"/>
+          <t>[Team/Contact](https://cre.vc)</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Sub-Saharan Africa focus</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>EchoVC</t>
+          <t>TLcom Capital</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Eghosa Omoigui</t>
+          <t>Maurizio Caio</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/pub/eghosa-omoigui/0/a/888</t>
+          <t>https://www.linkedin.com/in/mauriziocaio</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>[echovc.com](https://www.echovc.com)</t>
+          <t>[tlcomcapital.com](https://tlcomcapital.com)</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>UK / Kenya</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Africa / Emerging Markets</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Tech</t>
+          <t>Tech / Emerging Markets</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -1023,41 +1002,45 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Seed / Early Stage</t>
+          <t>Seed / Series A-Z</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>https://www.echovc.com/team</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr"/>
+          <t>[Team/Contact](https://tlcomcapital.com/team/)</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>African tech ecosystem</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Launch Africa</t>
+          <t>Novastar Ventures</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Zachariah George</t>
+          <t>Steve Beck</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/zachariahgeorge/</t>
+          <t>https://www.linkedin.com/in/stevebeck</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>[launchafrica.vc](https://launchafrica.vc)</t>
+          <t>[novastarventures.com](https://novastarventures.com)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Mauritius</t>
+          <t>Kenya</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1077,69 +1060,77 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Seed / Pre-Series A</t>
+          <t>Seed / Series A</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>https://www.launchafrica.vc/team</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr"/>
+          <t>[Team/Contact](https://novastarventures.com/team/)</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>East and West Africa</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Savannah Fund</t>
+          <t>Flat6Labs</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Mbwana Alliy</t>
+          <t>Ramez El-Serafy</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/mbwana/</t>
+          <t>https://www.linkedin.com/in/ramezelserafy</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>[savannah.vc](https://savannah.vc)</t>
+          <t>[flat6labs.com](https://flat6labs.com)</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Kenya</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>MENA</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Tech</t>
+          <t>Tech / Emerging Markets</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>VC</t>
+          <t>VC/Accelerator</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Seed</t>
+          <t>Pre-Seed / Seed</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>https://savannah.vc/team</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr"/>
+          <t>[Team/Contact](https://flat6labs.com/about/)</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>MENA region focus</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:L12"/>

</xml_diff>

<commit_message>
fix: enhance registry automation, data preservation, and path handling
- Updated `send_registry_emails.py` with robust, location-aware path resolution for environment and configuration files.
- Renamed internal path variables for better clarity.
- Enhanced `tender_sync_api.py` to fetch tenders for a rolling 7-day window.
- Updated `tender-sync.yml` workflow to run weekly on Mondays.
- Improved tender metadata capture: now uses the first available document link as the "Applying Link".
- Implemented automated cleanup of expired grants in `02_grants/`.
- Updated `md_to_excel.py` to preserve detailed descriptions for both grants and tenders in the final reports.
</commit_message>
<xml_diff>
--- a/published/01_Equity_Africa.xlsx
+++ b/published/01_Equity_Africa.xlsx
@@ -19,16 +19,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -55,7 +52,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -63,19 +60,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -526,33 +517,33 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Partech</t>
+          <t>Future Africa</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Philippe Collombel</t>
+          <t>Iyinoluwa Aboyeji</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/philippecollombel</t>
+          <t>https://www.linkedin.com/in/eaboyeji/</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[partechpartners.com](https://partechpartners.com)</t>
+          <t>[future.africa](https://www.future.africa)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Europe / Africa</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -567,55 +558,51 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Seed / Series A-Z</t>
+          <t>Seed / Series A</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>[Team/Contact](https://partechpartners.com/team/)</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>Strong Africa presence</t>
-        </is>
-      </c>
+          <t>https://www.future.africa/about-us</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Norrsken VC</t>
+          <t>Ventures Platform</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Niklas Adalberth</t>
+          <t>Kola Aina</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/niklas-adalberth</t>
+          <t>https://www.linkedin.com/in/kola-aina-vp/</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>[norrsken.vc](https://norrsken.vc)</t>
+          <t>[venturesplatform.com](https://www.venturesplatform.com)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Europe / Africa</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Tech / Impact / Emerging Markets</t>
+          <t>Tech / Fintech</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -630,50 +617,46 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>[Team/Contact](https://norrsken.vc/about)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Impact investing</t>
-        </is>
-      </c>
+          <t>https://www.venturesplatform.com/team</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>CRE Venture Capital</t>
+          <t>EchoVC</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Pardon Makumbe</t>
+          <t>Eghosa Omoigui</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/pardonmakumbe</t>
+          <t>https://www.linkedin.com/pub/eghosa-omoigui/0/a/888</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>[cre.vc](https://cre.vc)</t>
+          <t>[echovc.com](https://www.echovc.com)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>Africa / Emerging Markets</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Tech / Emerging Markets</t>
+          <t>Tech</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -683,45 +666,41 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Seed / Series A</t>
+          <t>Seed / Early Stage</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>[Team/Contact](https://cre.vc)</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>Sub-Saharan Africa focus</t>
-        </is>
-      </c>
+          <t>https://www.echovc.com/team</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TLcom Capital</t>
+          <t>Launch Africa</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Maurizio Caio</t>
+          <t>Zachariah George</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/mauriziocaio</t>
+          <t>https://www.linkedin.com/in/zachariahgeorge/</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>[tlcomcapital.com](https://tlcomcapital.com)</t>
+          <t>[launchafrica.vc](https://launchafrica.vc)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>UK / Kenya</t>
+          <t>Mauritius</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -741,40 +720,36 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Seed / Series A-Z</t>
+          <t>Seed / Pre-Series A</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>[Team/Contact](https://tlcomcapital.com/team/)</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>African tech ecosystem</t>
-        </is>
-      </c>
+          <t>https://www.launchafrica.vc/team</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Novastar Ventures</t>
+          <t>Savannah Fund</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Steve Beck</t>
+          <t>Mbwana Alliy</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/stevebeck</t>
+          <t>https://www.linkedin.com/in/mbwana/</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>[novastarventures.com](https://novastarventures.com)</t>
+          <t>[savannah.vc](https://savannah.vc)</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -789,7 +764,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Tech / Emerging Markets</t>
+          <t>Tech</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -799,50 +774,46 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Seed / Series A</t>
+          <t>Seed</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>[Team/Contact](https://novastarventures.com/team/)</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>East and West Africa</t>
-        </is>
-      </c>
+          <t>https://savannah.vc/team</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Flat6Labs</t>
+          <t>Ingressive Capital</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Ramez El-Serafy</t>
+          <t>Maya Horgan Famodu</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/ramezelserafy</t>
+          <t>https://www.linkedin.com/in/mayahorganfamodu</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>[flat6labs.com](https://flat6labs.com)</t>
+          <t>[ingressivecapital.com](https://ingressivecapital.com)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>MENA</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -852,50 +823,46 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>VC/Accelerator</t>
+          <t>VC</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Pre-Seed / Seed</t>
+          <t>Seed</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>[Team/Contact](https://flat6labs.com/about/)</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>MENA region focus</t>
-        </is>
-      </c>
+          <t>https://www.ingressivecapital.com/team</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Future Africa</t>
+          <t>4Di Capital</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Iyinoluwa Aboyeji</t>
+          <t>Justin Stanford</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/eaboyeji/</t>
+          <t>https://www.linkedin.com/in/justinstanford</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>[future.africa](https://www.future.africa)</t>
+          <t>[4dicapital.com](https://4dicapital.com)</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -905,7 +872,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Tech / Emerging Markets</t>
+          <t>Tech / Fintech</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -920,7 +887,7 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>https://www.future.africa/about-us</t>
+          <t>https://www.4dicapital.com/team</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr"/>
@@ -928,28 +895,28 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Ventures Platform</t>
+          <t>Knife Capital</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Kola Aina</t>
+          <t>Keet van Zyl</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/kola-aina-vp/</t>
+          <t>https://www.linkedin.com/in/keetvanzyl</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>[venturesplatform.com](https://www.venturesplatform.com)</t>
+          <t>[knifecap.com](https://knifecap.com)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -959,7 +926,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Tech / Fintech</t>
+          <t>Tech / Emerging Markets</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -969,12 +936,12 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Seed / Series A</t>
+          <t>Series A-B</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>https://www.venturesplatform.com/team</t>
+          <t>https://www.knifecap.com/team</t>
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
@@ -982,38 +949,38 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>EchoVC</t>
+          <t>Verod-Kepple Africa Ventures</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Eghosa Omoigui</t>
+          <t>Satoshi Akimoto</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/pub/eghosa-omoigui/0/a/888</t>
+          <t>https://www.linkedin.com/in/satoshi-akimoto-2b1b2a</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>[echovc.com](https://www.echovc.com)</t>
+          <t>[vkav.vc](https://vkav.vc)</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>Nigeria / Kenya</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Africa / Emerging Markets</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Tech</t>
+          <t>Tech / Fintech</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -1023,12 +990,12 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Seed / Early Stage</t>
+          <t>Series A-B</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>https://www.echovc.com/team</t>
+          <t>https://vkav.vc/team</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr"/>
@@ -1036,28 +1003,28 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Launch Africa</t>
+          <t>Microtraction</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Zachariah George</t>
+          <t>Yele Bademosi</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/zachariahgeorge/</t>
+          <t>https://www.linkedin.com/in/bademosiy</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>[launchafrica.vc](https://launchafrica.vc)</t>
+          <t>[microtraction.com](https://microtraction.com)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Mauritius</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1067,7 +1034,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Tech / Emerging Markets</t>
+          <t>Tech / Fintech</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1077,12 +1044,12 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Seed / Pre-Series A</t>
+          <t>Pre-Seed</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>https://www.launchafrica.vc/team</t>
+          <t>https://www.microtraction.com/team</t>
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
@@ -1090,28 +1057,28 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Savannah Fund</t>
+          <t>Kalon Venture Partners</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Mbwana Alliy</t>
+          <t>Clive Butkow</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/mbwana/</t>
+          <t>https://www.linkedin.com/in/clivebutkow</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>[savannah.vc](https://savannah.vc)</t>
+          <t>[kalonvp.com](https://kalonvp.com)</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Kenya</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1121,7 +1088,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Tech</t>
+          <t>Tech / AI / SaaS</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1131,12 +1098,12 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Seed</t>
+          <t>Seed / Series A</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>https://savannah.vc/team</t>
+          <t>https://kalonvp.com/team</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr"/>
@@ -1144,28 +1111,28 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Ingressive Capital</t>
+          <t>Savant</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Maya Horgan Famodu</t>
+          <t>Nick Allen</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/mayahorganfamodu</t>
+          <t>https://www.linkedin.com/in/nick-allen-2b1b2a</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>[ingressivecapital.com](https://ingressivecapital.com)</t>
+          <t>[savant.co.za](https://savant.co.za)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1175,12 +1142,12 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Tech / Emerging Markets</t>
+          <t>DeepTech / Tech</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>VC</t>
+          <t>VC / Incubator</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1190,7 +1157,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>https://www.ingressivecapital.com/team</t>
+          <t>https://savant.co.za/team</t>
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
@@ -1198,28 +1165,28 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>4Di Capital</t>
+          <t>Adlevo Capital</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Justin Stanford</t>
+          <t>Yemi Lalude</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/justinstanford</t>
+          <t>https://www.linkedin.com/in/yemilalude</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>[4dicapital.com](https://4dicapital.com)</t>
+          <t>[adlevocapital.com](https://adlevocapital.com)</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Nigeria / Mauritius</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1229,22 +1196,22 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Tech / Fintech</t>
+          <t>Tech</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>VC</t>
+          <t>VC / PE</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Seed / Series A</t>
+          <t>Series A-Z</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>https://www.4dicapital.com/team</t>
+          <t>https://adlevocapital.com/team</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr"/>
@@ -1252,33 +1219,33 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Knife Capital</t>
+          <t>Partech</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Keet van Zyl</t>
+          <t>Philippe Collombel</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/keetvanzyl</t>
+          <t>https://www.linkedin.com/in/philippecollombel</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>[knifecap.com](https://knifecap.com)</t>
+          <t>[partechpartners.com](https://partechpartners.com)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>France</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>Europe / Africa</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1293,51 +1260,55 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Series A-B</t>
+          <t>Seed / Series A-Z</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>https://www.knifecap.com/team</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr"/>
+          <t>[Team/Contact](https://partechpartners.com/team/)</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Strong Africa presence</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Verod-Kepple Africa Ventures</t>
+          <t>Norrsken VC</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Satoshi Akimoto</t>
+          <t>Niklas Adalberth</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/satoshi-akimoto-2b1b2a</t>
+          <t>https://www.linkedin.com/in/niklas-adalberth</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>[vkav.vc](https://vkav.vc)</t>
+          <t>[norrsken.vc](https://norrsken.vc)</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Nigeria / Kenya</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>Europe / Africa</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Tech / Fintech</t>
+          <t>Tech / Impact / Emerging Markets</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1347,41 +1318,45 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Series A-B</t>
+          <t>Seed / Series A</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>https://vkav.vc/team</t>
-        </is>
-      </c>
-      <c r="L16" s="2" t="inlineStr"/>
+          <t>[Team/Contact](https://norrsken.vc/about)</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Impact investing</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Microtraction</t>
+          <t>CRE Venture Capital</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Yele Bademosi</t>
+          <t>Pardon Makumbe</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/bademosiy</t>
+          <t>https://www.linkedin.com/in/pardonmakumbe</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>[microtraction.com](https://microtraction.com)</t>
+          <t>[cre.vc](https://cre.vc)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1391,7 +1366,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Tech / Fintech</t>
+          <t>Tech / Emerging Markets</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1401,41 +1376,45 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Pre-Seed</t>
+          <t>Seed / Series A</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>https://www.microtraction.com/team</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr"/>
+          <t>[Team/Contact](https://cre.vc)</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Sub-Saharan Africa focus</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Kalon Venture Partners</t>
+          <t>TLcom Capital</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Clive Butkow</t>
+          <t>Maurizio Caio</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/clivebutkow</t>
+          <t>https://www.linkedin.com/in/mauriziocaio</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>[kalonvp.com](https://kalonvp.com)</t>
+          <t>[tlcomcapital.com](https://tlcomcapital.com)</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>UK / Kenya</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1445,7 +1424,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Tech / AI / SaaS</t>
+          <t>Tech / Emerging Markets</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -1455,41 +1434,45 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Seed / Series A</t>
+          <t>Seed / Series A-Z</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>https://kalonvp.com/team</t>
-        </is>
-      </c>
-      <c r="L18" s="2" t="inlineStr"/>
+          <t>[Team/Contact](https://tlcomcapital.com/team/)</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>African tech ecosystem</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Savant</t>
+          <t>Novastar Ventures</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Nick Allen</t>
+          <t>Steve Beck</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/nick-allen-2b1b2a</t>
+          <t>https://www.linkedin.com/in/stevebeck</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>[savant.co.za](https://savant.co.za)</t>
+          <t>[novastarventures.com](https://novastarventures.com)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Kenya</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1499,79 +1482,87 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>DeepTech / Tech</t>
+          <t>Tech / Emerging Markets</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>VC / Incubator</t>
+          <t>VC</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Seed</t>
+          <t>Seed / Series A</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>https://savant.co.za/team</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr"/>
+          <t>[Team/Contact](https://novastarventures.com/team/)</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>East and West Africa</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Adlevo Capital</t>
+          <t>Flat6Labs</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Yemi Lalude</t>
+          <t>Ramez El-Serafy</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/yemilalude</t>
+          <t>https://www.linkedin.com/in/ramezelserafy</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>[adlevocapital.com](https://adlevocapital.com)</t>
+          <t>[flat6labs.com](https://flat6labs.com)</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Nigeria / Mauritius</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>MENA</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Tech</t>
+          <t>Tech / Emerging Markets</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>VC / PE</t>
+          <t>VC/Accelerator</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>Series A-Z</t>
+          <t>Pre-Seed / Seed</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>https://adlevocapital.com/team</t>
-        </is>
-      </c>
-      <c r="L20" s="2" t="inlineStr"/>
+          <t>[Team/Contact](https://flat6labs.com/about/)</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>MENA region focus</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:L20"/>

</xml_diff>

<commit_message>
fix: upgrade registry automation for data integrity and multi-format reporting
- **Data Integrity**: `tender_sync_api.py` now skips overwriting any files marked as 'VERIFIED' to preserve manual steward effort.
- **Reporting**: `md_to_excel.py` now generates both Excel and PDF versions of all reports using `reportlab`.
- **Transparency**: Published reports now hide internal fields like 'Source' and 'Verification Status' for a cleaner professional look.
- **Improved Metadata**:
  - Tender 'Applying Link' renamed to 'Direct Link'.
  - Added support for extracting and reporting ALL document links found in tender cards.
  - Preserved detailed descriptions in both Excel and PDF outputs.
- **Workflow Optimization**: Aligned all registry automation schedules to run weekly (Mondays) and added necessary dependencies for PDF generation.
- **Refinement**: Updated tender template AI checklist with more specific document analysis tasks.
</commit_message>
<xml_diff>
--- a/published/01_Equity_Africa.xlsx
+++ b/published/01_Equity_Africa.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Africa_Focus" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Africa_Focus'!$A$1:$L$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Africa_Focus'!$A$1:$K$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -448,8 +448,7 @@
     <col width="34" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="21" customWidth="1" min="10" max="10"/>
-    <col width="50" customWidth="1" min="11" max="11"/>
-    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -505,11 +504,6 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Source / Verification</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
           <t>Notes</t>
         </is>
       </c>
@@ -561,12 +555,7 @@
           <t>Seed / Series A</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.future.africa/about-us</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -615,12 +604,7 @@
           <t>Seed / Series A</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>https://www.venturesplatform.com/team</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -669,12 +653,7 @@
           <t>Seed / Early Stage</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>https://www.echovc.com/team</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -723,12 +702,7 @@
           <t>Seed / Pre-Series A</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>https://www.launchafrica.vc/team</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -777,12 +751,7 @@
           <t>Seed</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>https://savannah.vc/team</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -831,12 +800,7 @@
           <t>Seed</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>https://www.ingressivecapital.com/team</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -885,12 +849,7 @@
           <t>Seed / Series A</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>https://www.4dicapital.com/team</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -939,12 +898,7 @@
           <t>Series A-B</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>https://www.knifecap.com/team</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -993,12 +947,7 @@
           <t>Series A-B</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>https://vkav.vc/team</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1047,12 +996,7 @@
           <t>Pre-Seed</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>https://www.microtraction.com/team</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1101,12 +1045,7 @@
           <t>Seed / Series A</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>https://kalonvp.com/team</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1155,12 +1094,7 @@
           <t>Seed</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>https://savant.co.za/team</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1209,12 +1143,7 @@
           <t>Series A-Z</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>https://adlevocapital.com/team</t>
-        </is>
-      </c>
-      <c r="L14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1265,11 +1194,6 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>[Team/Contact](https://partechpartners.com/team/)</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
           <t>Strong Africa presence</t>
         </is>
       </c>
@@ -1323,11 +1247,6 @@
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>[Team/Contact](https://norrsken.vc/about)</t>
-        </is>
-      </c>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
           <t>Impact investing</t>
         </is>
       </c>
@@ -1381,11 +1300,6 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>[Team/Contact](https://cre.vc)</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
           <t>Sub-Saharan Africa focus</t>
         </is>
       </c>
@@ -1439,11 +1353,6 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>[Team/Contact](https://tlcomcapital.com/team/)</t>
-        </is>
-      </c>
-      <c r="L18" s="2" t="inlineStr">
-        <is>
           <t>African tech ecosystem</t>
         </is>
       </c>
@@ -1497,11 +1406,6 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>[Team/Contact](https://novastarventures.com/team/)</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
           <t>East and West Africa</t>
         </is>
       </c>
@@ -1555,17 +1459,12 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>[Team/Contact](https://flat6labs.com/about/)</t>
-        </is>
-      </c>
-      <c r="L20" s="2" t="inlineStr">
-        <is>
           <t>MENA region focus</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L20"/>
+  <autoFilter ref="A1:K20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: resolve missing dependencies and workflow inconsistencies
- Added `python-dotenv` and `pycryptodome` to `registry-sync-excel.yml`, `tender-sync.yml`, and `registry-weekly-report.yml`.
- Standardized environment loading across all scripts to ensure consistent parsing of monorepo secrets.
- Verified that all registry automation workflows now include the necessary cryptographic libraries for reversible privacy.
</commit_message>
<xml_diff>
--- a/published/01_Equity_Africa.xlsx
+++ b/published/01_Equity_Africa.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Africa_Focus" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Africa_Focus'!$A$1:$L$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Africa_Focus'!$A$1:$K$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,16 +19,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -55,7 +52,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -63,19 +60,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -444,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -457,8 +448,7 @@
     <col width="34" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="21" customWidth="1" min="10" max="10"/>
-    <col width="50" customWidth="1" min="11" max="11"/>
-    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -514,11 +504,6 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Source / Verification</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
           <t>Notes</t>
         </is>
       </c>
@@ -526,33 +511,33 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Partech</t>
+          <t>Future Africa</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Philippe Collombel</t>
+          <t>Iyinoluwa Aboyeji</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/philippecollombel</t>
+          <t>https://www.linkedin.com/in/eaboyeji/</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[partechpartners.com](https://partechpartners.com)</t>
+          <t>[future.africa](https://www.future.africa)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Europe / Africa</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -567,55 +552,46 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Seed / Series A-Z</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>[Team/Contact](https://partechpartners.com/team/)</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>Strong Africa presence</t>
-        </is>
-      </c>
+          <t>Seed / Series A</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Norrsken VC</t>
+          <t>Ventures Platform</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Niklas Adalberth</t>
+          <t>Kola Aina</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/niklas-adalberth</t>
+          <t>https://www.linkedin.com/in/kola-aina-vp/</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>[norrsken.vc](https://norrsken.vc)</t>
+          <t>[venturesplatform.com](https://www.venturesplatform.com)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Europe / Africa</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Tech / Impact / Emerging Markets</t>
+          <t>Tech / Fintech</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -628,52 +604,43 @@
           <t>Seed / Series A</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>[Team/Contact](https://norrsken.vc/about)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Impact investing</t>
-        </is>
-      </c>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>CRE Venture Capital</t>
+          <t>EchoVC</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Pardon Makumbe</t>
+          <t>Eghosa Omoigui</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/pardonmakumbe</t>
+          <t>https://www.linkedin.com/pub/eghosa-omoigui/0/a/888</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>[cre.vc](https://cre.vc)</t>
+          <t>[echovc.com](https://www.echovc.com)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>Africa / Emerging Markets</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Tech / Emerging Markets</t>
+          <t>Tech</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -683,45 +650,36 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Seed / Series A</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>[Team/Contact](https://cre.vc)</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>Sub-Saharan Africa focus</t>
-        </is>
-      </c>
+          <t>Seed / Early Stage</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TLcom Capital</t>
+          <t>Launch Africa</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Maurizio Caio</t>
+          <t>Zachariah George</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/mauriziocaio</t>
+          <t>https://www.linkedin.com/in/zachariahgeorge/</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>[tlcomcapital.com](https://tlcomcapital.com)</t>
+          <t>[launchafrica.vc](https://launchafrica.vc)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>UK / Kenya</t>
+          <t>Mauritius</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -741,40 +699,31 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Seed / Series A-Z</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>[Team/Contact](https://tlcomcapital.com/team/)</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>African tech ecosystem</t>
-        </is>
-      </c>
+          <t>Seed / Pre-Series A</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Novastar Ventures</t>
+          <t>Savannah Fund</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Steve Beck</t>
+          <t>Mbwana Alliy</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/stevebeck</t>
+          <t>https://www.linkedin.com/in/mbwana/</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>[novastarventures.com](https://novastarventures.com)</t>
+          <t>[savannah.vc](https://savannah.vc)</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -789,7 +738,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Tech / Emerging Markets</t>
+          <t>Tech</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -799,50 +748,41 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Seed / Series A</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>[Team/Contact](https://novastarventures.com/team/)</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>East and West Africa</t>
-        </is>
-      </c>
+          <t>Seed</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Flat6Labs</t>
+          <t>Ingressive Capital</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Ramez El-Serafy</t>
+          <t>Maya Horgan Famodu</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/ramezelserafy</t>
+          <t>https://www.linkedin.com/in/mayahorganfamodu</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>[flat6labs.com](https://flat6labs.com)</t>
+          <t>[ingressivecapital.com](https://ingressivecapital.com)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>MENA</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -852,50 +792,41 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>VC/Accelerator</t>
+          <t>VC</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Pre-Seed / Seed</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>[Team/Contact](https://flat6labs.com/about/)</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>MENA region focus</t>
-        </is>
-      </c>
+          <t>Seed</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Future Africa</t>
+          <t>4Di Capital</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Iyinoluwa Aboyeji</t>
+          <t>Justin Stanford</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/eaboyeji/</t>
+          <t>https://www.linkedin.com/in/justinstanford</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>[future.africa](https://www.future.africa)</t>
+          <t>[4dicapital.com](https://4dicapital.com)</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -905,7 +836,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Tech / Emerging Markets</t>
+          <t>Tech / Fintech</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -918,38 +849,33 @@
           <t>Seed / Series A</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>https://www.future.africa/about-us</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Ventures Platform</t>
+          <t>Knife Capital</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Kola Aina</t>
+          <t>Keet van Zyl</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/kola-aina-vp/</t>
+          <t>https://www.linkedin.com/in/keetvanzyl</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>[venturesplatform.com](https://www.venturesplatform.com)</t>
+          <t>[knifecap.com](https://knifecap.com)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -959,7 +885,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Tech / Fintech</t>
+          <t>Tech / Emerging Markets</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -969,51 +895,46 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Seed / Series A</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>https://www.venturesplatform.com/team</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr"/>
+          <t>Series A-B</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>EchoVC</t>
+          <t>Verod-Kepple Africa Ventures</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Eghosa Omoigui</t>
+          <t>Satoshi Akimoto</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/pub/eghosa-omoigui/0/a/888</t>
+          <t>https://www.linkedin.com/in/satoshi-akimoto-2b1b2a</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>[echovc.com](https://www.echovc.com)</t>
+          <t>[vkav.vc](https://vkav.vc)</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>Nigeria / Kenya</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Africa / Emerging Markets</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Tech</t>
+          <t>Tech / Fintech</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -1023,41 +944,36 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Seed / Early Stage</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>https://www.echovc.com/team</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr"/>
+          <t>Series A-B</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Launch Africa</t>
+          <t>Microtraction</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Zachariah George</t>
+          <t>Yele Bademosi</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/zachariahgeorge/</t>
+          <t>https://www.linkedin.com/in/bademosiy</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>[launchafrica.vc](https://launchafrica.vc)</t>
+          <t>[microtraction.com](https://microtraction.com)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Mauritius</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1067,7 +983,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Tech / Emerging Markets</t>
+          <t>Tech / Fintech</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1077,41 +993,36 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Seed / Pre-Series A</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>https://www.launchafrica.vc/team</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr"/>
+          <t>Pre-Seed</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Savannah Fund</t>
+          <t>Kalon Venture Partners</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Mbwana Alliy</t>
+          <t>Clive Butkow</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/mbwana/</t>
+          <t>https://www.linkedin.com/in/clivebutkow</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>[savannah.vc](https://savannah.vc)</t>
+          <t>[kalonvp.com](https://kalonvp.com)</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Kenya</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1121,7 +1032,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Tech</t>
+          <t>Tech / AI / SaaS</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1131,41 +1042,36 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Seed</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>https://savannah.vc/team</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr"/>
+          <t>Seed / Series A</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Ingressive Capital</t>
+          <t>Savant</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Maya Horgan Famodu</t>
+          <t>Nick Allen</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/mayahorganfamodu</t>
+          <t>https://www.linkedin.com/in/nick-allen-2b1b2a</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>[ingressivecapital.com](https://ingressivecapital.com)</t>
+          <t>[savant.co.za](https://savant.co.za)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1175,12 +1081,12 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Tech / Emerging Markets</t>
+          <t>DeepTech / Tech</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>VC</t>
+          <t>VC / Incubator</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1188,38 +1094,33 @@
           <t>Seed</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>https://www.ingressivecapital.com/team</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>4Di Capital</t>
+          <t>Adlevo Capital</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Justin Stanford</t>
+          <t>Yemi Lalude</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/justinstanford</t>
+          <t>https://www.linkedin.com/in/yemilalude</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>[4dicapital.com](https://4dicapital.com)</t>
+          <t>[adlevocapital.com](https://adlevocapital.com)</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Nigeria / Mauritius</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1229,56 +1130,51 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Tech / Fintech</t>
+          <t>Tech</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>VC</t>
+          <t>VC / PE</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Seed / Series A</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>https://www.4dicapital.com/team</t>
-        </is>
-      </c>
-      <c r="L14" s="2" t="inlineStr"/>
+          <t>Series A-Z</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Knife Capital</t>
+          <t>Partech</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Keet van Zyl</t>
+          <t>Philippe Collombel</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/keetvanzyl</t>
+          <t>https://www.linkedin.com/in/philippecollombel</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>[knifecap.com](https://knifecap.com)</t>
+          <t>[partechpartners.com](https://partechpartners.com)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>France</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>Europe / Africa</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1293,51 +1189,50 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Series A-B</t>
+          <t>Seed / Series A-Z</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>https://www.knifecap.com/team</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr"/>
+          <t>Strong Africa presence</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Verod-Kepple Africa Ventures</t>
+          <t>Norrsken VC</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Satoshi Akimoto</t>
+          <t>Niklas Adalberth</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/satoshi-akimoto-2b1b2a</t>
+          <t>https://www.linkedin.com/in/niklas-adalberth</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>[vkav.vc](https://vkav.vc)</t>
+          <t>[norrsken.vc](https://norrsken.vc)</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Nigeria / Kenya</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>Europe / Africa</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Tech / Fintech</t>
+          <t>Tech / Impact / Emerging Markets</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1347,41 +1242,40 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Series A-B</t>
+          <t>Seed / Series A</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>https://vkav.vc/team</t>
-        </is>
-      </c>
-      <c r="L16" s="2" t="inlineStr"/>
+          <t>Impact investing</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Microtraction</t>
+          <t>CRE Venture Capital</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Yele Bademosi</t>
+          <t>Pardon Makumbe</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/bademosiy</t>
+          <t>https://www.linkedin.com/in/pardonmakumbe</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>[microtraction.com](https://microtraction.com)</t>
+          <t>[cre.vc](https://cre.vc)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1391,7 +1285,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Tech / Fintech</t>
+          <t>Tech / Emerging Markets</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1401,41 +1295,40 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Pre-Seed</t>
+          <t>Seed / Series A</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>https://www.microtraction.com/team</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr"/>
+          <t>Sub-Saharan Africa focus</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Kalon Venture Partners</t>
+          <t>TLcom Capital</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Clive Butkow</t>
+          <t>Maurizio Caio</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/clivebutkow</t>
+          <t>https://www.linkedin.com/in/mauriziocaio</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>[kalonvp.com](https://kalonvp.com)</t>
+          <t>[tlcomcapital.com](https://tlcomcapital.com)</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>UK / Kenya</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1445,7 +1338,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Tech / AI / SaaS</t>
+          <t>Tech / Emerging Markets</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -1455,41 +1348,40 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Seed / Series A</t>
+          <t>Seed / Series A-Z</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>https://kalonvp.com/team</t>
-        </is>
-      </c>
-      <c r="L18" s="2" t="inlineStr"/>
+          <t>African tech ecosystem</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Savant</t>
+          <t>Novastar Ventures</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Nick Allen</t>
+          <t>Steve Beck</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/nick-allen-2b1b2a</t>
+          <t>https://www.linkedin.com/in/stevebeck</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>[savant.co.za](https://savant.co.za)</t>
+          <t>[novastarventures.com](https://novastarventures.com)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Kenya</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1499,82 +1391,80 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>DeepTech / Tech</t>
+          <t>Tech / Emerging Markets</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>VC / Incubator</t>
+          <t>VC</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Seed</t>
+          <t>Seed / Series A</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>https://savant.co.za/team</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr"/>
+          <t>East and West Africa</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Adlevo Capital</t>
+          <t>Flat6Labs</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Yemi Lalude</t>
+          <t>Ramez El-Serafy</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/yemilalude</t>
+          <t>https://www.linkedin.com/in/ramezelserafy</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>[adlevocapital.com](https://adlevocapital.com)</t>
+          <t>[flat6labs.com](https://flat6labs.com)</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Nigeria / Mauritius</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>MENA</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Tech</t>
+          <t>Tech / Emerging Markets</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>VC / PE</t>
+          <t>VC/Accelerator</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>Series A-Z</t>
+          <t>Pre-Seed / Seed</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>https://adlevocapital.com/team</t>
-        </is>
-      </c>
-      <c r="L20" s="2" t="inlineStr"/>
+          <t>MENA region focus</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L20"/>
+  <autoFilter ref="A1:K20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>